<commit_message>
Dormitorio suite: la interior es SO; el resto de las orientaciones queda pendiente
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -4418,7 +4418,7 @@
       <c r="A156" s="47" t="n"/>
       <c r="B156" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C156" s="18" t="inlineStr">
@@ -4464,7 +4464,7 @@
       <c r="A158" s="47" t="n"/>
       <c r="B158" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C158" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Dormitorio suite: aislada NE, SO (VA01) y NO; interior SE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -4418,7 +4418,7 @@
       <c r="A156" s="47" t="n"/>
       <c r="B156" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C156" s="18" t="inlineStr">
@@ -4441,7 +4441,7 @@
       <c r="A157" s="47" t="n"/>
       <c r="B157" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (NO)</t>
         </is>
       </c>
       <c r="C157" s="18" t="inlineStr">
@@ -4464,7 +4464,7 @@
       <c r="A158" s="47" t="n"/>
       <c r="B158" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (SO)</t>
+          <t>INTERIORES (SE)</t>
         </is>
       </c>
       <c r="C158" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Bano suite: las dos interiores de 1,72 son NO y SE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -4991,7 +4991,7 @@
       <c r="A187" s="47" t="n"/>
       <c r="B187" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C187" s="18" t="inlineStr">
@@ -5037,7 +5037,7 @@
       <c r="A189" s="50" t="n"/>
       <c r="B189" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SE)</t>
         </is>
       </c>
       <c r="C189" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Bano suite: lindes con el dormitorio suite y el bano de visitas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -4991,7 +4991,7 @@
       <c r="A187" s="47" t="n"/>
       <c r="B187" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NO)</t>
+          <t>INTERIORES (NO, dormitorio suite)</t>
         </is>
       </c>
       <c r="C187" s="18" t="inlineStr">
@@ -5037,7 +5037,7 @@
       <c r="A189" s="50" t="n"/>
       <c r="B189" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (SE)</t>
+          <t>INTERIORES (SE, bano visitas)</t>
         </is>
       </c>
       <c r="C189" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Bano suite: la SE da al dormitorio suite y la NO al bano de visitas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -4991,7 +4991,7 @@
       <c r="A187" s="47" t="n"/>
       <c r="B187" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NO, dormitorio suite)</t>
+          <t>INTERIORES (NO, bano visitas)</t>
         </is>
       </c>
       <c r="C187" s="18" t="inlineStr">
@@ -5037,7 +5037,7 @@
       <c r="A189" s="50" t="n"/>
       <c r="B189" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (SE, bano visitas)</t>
+          <t>INTERIORES (SE, dormitorio suite)</t>
         </is>
       </c>
       <c r="C189" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Dormitorio suite: la ciega es SE (frente) y la interior NO
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -4441,7 +4441,7 @@
       <c r="A157" s="47" t="n"/>
       <c r="B157" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (NO)</t>
+          <t>AISLADAS (SE)</t>
         </is>
       </c>
       <c r="C157" s="18" t="inlineStr">
@@ -4464,7 +4464,7 @@
       <c r="A158" s="47" t="n"/>
       <c r="B158" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (SE)</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C158" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Vestidor: lado largo SO (hacia el hall) y tramos de 3,38 y 1,49 al NE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -3264,7 +3264,7 @@
       <c r="A96" s="43" t="n"/>
       <c r="B96" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C96" s="18" t="inlineStr">
@@ -3302,7 +3302,7 @@
       <c r="A98" s="47" t="n"/>
       <c r="B98" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C98" s="18" t="inlineStr">
@@ -3348,7 +3348,7 @@
       <c r="A100" s="47" t="n"/>
       <c r="B100" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C100" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Escalera: la aislada de 4,06 es NE y la interior SO
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -3868,7 +3868,7 @@
       <c r="A128" s="43" t="n"/>
       <c r="B128" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C128" s="18" t="inlineStr">
@@ -3891,7 +3891,7 @@
       <c r="A129" s="47" t="n"/>
       <c r="B129" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS (SO)</t>
+          <t>AISLADAS</t>
         </is>
       </c>
       <c r="C129" s="18" t="inlineStr">
@@ -3914,7 +3914,7 @@
       <c r="A130" s="47" t="n"/>
       <c r="B130" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C130" s="18" t="inlineStr">
@@ -3937,7 +3937,7 @@
       <c r="A131" s="50" t="n"/>
       <c r="B131" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (NE)</t>
+          <t>INTERIORES</t>
         </is>
       </c>
       <c r="C131" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Escalera: la aislada de 1,73 es SE y la interior NO
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -3891,7 +3891,7 @@
       <c r="A129" s="47" t="n"/>
       <c r="B129" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SE)</t>
         </is>
       </c>
       <c r="C129" s="18" t="inlineStr">
@@ -3937,7 +3937,7 @@
       <c r="A131" s="50" t="n"/>
       <c r="B131" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C131" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Bano visitas: orientaciones de las cuatro paredes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -5480,7 +5480,7 @@
       <c r="A214" s="43" t="n"/>
       <c r="B214" s="79" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (NE)</t>
         </is>
       </c>
       <c r="C214" s="18" t="inlineStr">
@@ -5518,7 +5518,7 @@
       <c r="A216" s="47" t="n"/>
       <c r="B216" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C216" s="18" t="inlineStr">
@@ -5541,7 +5541,7 @@
       <c r="A217" s="47" t="n"/>
       <c r="B217" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SE, bano suite)</t>
         </is>
       </c>
       <c r="C217" s="18" t="inlineStr">
@@ -5564,7 +5564,7 @@
       <c r="A218" s="50" t="n"/>
       <c r="B218" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C218" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Balance termico: los rotulos de las paredes llevan solo la orientacion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -1684,7 +1684,7 @@
       <c r="A12" s="47" t="n"/>
       <c r="B12" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (SE, galeria y living)</t>
+          <t>INTERIORES (SE)</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
@@ -1707,7 +1707,7 @@
       <c r="A13" s="50" t="n"/>
       <c r="B13" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (NE, deposito y lavadero)</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -2242,7 +2242,7 @@
       <c r="A42" s="47" t="n"/>
       <c r="B42" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NE, cocina)</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
@@ -2265,7 +2265,7 @@
       <c r="A43" s="47" t="n"/>
       <c r="B43" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NO, galeria)</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
@@ -2288,7 +2288,7 @@
       <c r="A44" s="50" t="n"/>
       <c r="B44" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (SO, escalera y bano exterior)</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
@@ -2837,7 +2837,7 @@
       <c r="A73" s="47" t="n"/>
       <c r="B73" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NE, vestidor)</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C73" s="18" t="inlineStr">
@@ -2860,7 +2860,7 @@
       <c r="A74" s="50" t="n"/>
       <c r="B74" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (NO, living comedor)</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C74" s="18" t="inlineStr">
@@ -3302,7 +3302,7 @@
       <c r="A98" s="47" t="n"/>
       <c r="B98" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (SO, hall de ingreso)</t>
+          <t>INTERIORES (SO)</t>
         </is>
       </c>
       <c r="C98" s="18" t="inlineStr">
@@ -4968,7 +4968,7 @@
       <c r="A186" s="47" t="n"/>
       <c r="B186" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (NO, bano visitas)</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C186" s="18" t="inlineStr">
@@ -5014,7 +5014,7 @@
       <c r="A188" s="50" t="n"/>
       <c r="B188" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES (SE, dormitorio suite)</t>
+          <t>INTERIORES (SE)</t>
         </is>
       </c>
       <c r="C188" s="18" t="inlineStr">
@@ -5541,7 +5541,7 @@
       <c r="A217" s="47" t="n"/>
       <c r="B217" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES (SE, bano suite)</t>
+          <t>INTERIORES (SE)</t>
         </is>
       </c>
       <c r="C217" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Dormitorio Norte: la aislada de 4,00 es SO y la interior NE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -6107,7 +6107,7 @@
       <c r="A247" s="47" t="n"/>
       <c r="B247" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C247" s="18" t="inlineStr">
@@ -6130,7 +6130,7 @@
       <c r="A248" s="47" t="n"/>
       <c r="B248" s="81" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C248" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Dormitorio Sur: la ciega de 3,50 es SO y la interior NE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -7183,7 +7183,7 @@
       <c r="A305" s="47" t="n"/>
       <c r="B305" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SO)</t>
         </is>
       </c>
       <c r="C305" s="18" t="inlineStr">
@@ -7229,7 +7229,7 @@
       <c r="A307" s="50" t="n"/>
       <c r="B307" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NE)</t>
         </is>
       </c>
       <c r="C307" s="18" t="inlineStr">

</xml_diff>

<commit_message>
Bano 17: la aislada de 1,60 es SE y la interior NO; todas las paredes con orientacion
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -7726,7 +7726,7 @@
       <c r="A334" s="47" t="n"/>
       <c r="B334" s="81" t="inlineStr">
         <is>
-          <t>AISLADAS</t>
+          <t>AISLADAS (SE)</t>
         </is>
       </c>
       <c r="C334" s="18" t="inlineStr">
@@ -7772,7 +7772,7 @@
       <c r="A336" s="50" t="n"/>
       <c r="B336" s="82" t="inlineStr">
         <is>
-          <t>INTERIORES</t>
+          <t>INTERIORES (NO)</t>
         </is>
       </c>
       <c r="C336" s="18" t="inlineStr">

</xml_diff>

<commit_message>
PDF de cada planilla para insertar en AutoCAD; cada local del balance en su pagina
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/Balance termico (para AutoCAD).xlsx
+++ b/planillas/Balance termico (para AutoCAD).xlsx
@@ -8262,5 +8262,18 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
+  <rowBreaks count="11" manualBreakCount="11">
+    <brk id="33" min="0" max="16383" man="1"/>
+    <brk id="65" min="0" max="16383" man="1"/>
+    <brk id="92" min="0" max="16383" man="1"/>
+    <brk id="125" min="0" max="16383" man="1"/>
+    <brk id="151" min="0" max="16383" man="1"/>
+    <brk id="183" min="0" max="16383" man="1"/>
+    <brk id="214" min="0" max="16383" man="1"/>
+    <brk id="245" min="0" max="16383" man="1"/>
+    <brk id="277" min="0" max="16383" man="1"/>
+    <brk id="307" min="0" max="16383" man="1"/>
+    <brk id="337" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>